<commit_message>
Comparer les corridors Lomé et Cotonou et actualiser les taux
- nouvel onglet Corridors : quatre scénarios d'acheminement (Lomé prudent ou
  optimiste, Cotonou via le Nigeria, Cotonou frontière rouverte) pilotés par
  un sélecteur unique dans les hypothèses
- signale la fermeture de la frontière Bénin-Niger depuis juillet 2023, non
  levée en août 2026, et la réouverture du corridor Tsamiya-Kamba par le
  Nigeria le 9 février 2026
- PCS ramené à 0,8 % (taux appliqué au Niger) : droits à 7,3 % au lieu de 7,5 %
- prix de vente et tarif commercial recalculés
- note de calcul : tableau du niveau de fiabilité de chaque donnée, distinguant
  les chiffres fermes des fourchettes de marché et de ce qui reste à confirmer

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017KgrzJui3uU4u3uue6UcyC
</commit_message>
<xml_diff>
--- a/COMMERCIAL/2026-IMPORT-MACHINES-AGRICOLES-ZENO/PRIX_DE_REVIENT_ET_PRIX_DE_VENTE.xlsx
+++ b/COMMERCIAL/2026-IMPORT-MACHINES-AGRICOLES-ZENO/PRIX_DE_REVIENT_ET_PRIX_DE_VENTE.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothèses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prix de revient" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prix de vente" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corridors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prix de revient" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prix de vente" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,15 +20,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="#,##0 &quot;F&quot;"/>
-    <numFmt numFmtId="165" formatCode="#,##0.000"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00 &quot;$&quot;;(#,##0.00);-"/>
-    <numFmt numFmtId="167" formatCode="#,##0 &quot;F&quot;;(#,##0) &quot;F&quot;;-"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
+  <numFmts count="8">
+    <numFmt numFmtId="164" formatCode="#,##0.00 &quot;$&quot;;(#,##0.00);-"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;F&quot;;(#,##0) &quot;F&quot;;-"/>
+    <numFmt numFmtId="166" formatCode="#,##0 &quot;km&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0 &quot;j&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0 &quot;F&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +52,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000D3D6B"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -65,12 +68,34 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00606060"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000D3D6B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="000D3D6B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00606060"/>
       <sz val="9"/>
     </font>
     <font>
@@ -83,10 +108,6 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="9"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -97,7 +118,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFEFEF"/>
+        <fgColor rgb="001F4E9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +128,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E9C"/>
+        <fgColor rgb="00EFEFEF"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,71 +163,79 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -594,387 +623,410 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>► CORRIDOR RETENU (1 = Lomé prudent · 2 = Lomé optimiste · 3 = Cotonou via Nigeria · 4 = Cotonou frontière ouverte)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Voir l'onglet « Corridors » pour le détail et l'état de la frontière Bénin–Niger.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>1. CHANGE</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Taux de change  1 USD =</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="9" t="n">
         <v>560</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Moyenne 2026 : 559 XOF/USD (exchange-rates.org). 560 retenu par prudence.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2. EMBALLAGE (caisses bois export)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Coefficient de majoration du volume</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="10" t="n">
         <v>1.15</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Caisse bois : +15 % sur le volume machine.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Coefficient de majoration du poids</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="10" t="n">
         <v>1.12</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Caisse bois : +12 % sur le poids machine.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>3. LOGISTIQUE — 1 conteneur 20' (Qingdao → Lomé → Niamey)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Fret maritime Qingdao → Lomé, 20' FCL (USD)</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>1900</v>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Marché 2026 Chine → Lomé : 1 350 à 1 950 USD port à port, surcharges incluses.</t>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Fret maritime Qingdao → port de débarquement, 20' FCL (USD)</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
+        <f>INDEX(Corridors!$C$5:$F$5,1,'Hypothèses'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Piloté par le corridor retenu (onglet Corridors, ligne 1).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Fret maritime (FCFA)</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="12">
         <f>'Hypothèses'!B12*'Hypothèses'!B5</f>
         <v/>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Fret en dollars × taux de change</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Assurance transport (% de FOB + fret)</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="13" t="n">
         <v>0.005</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Police ad valorem usuelle : 0,4 à 0,7 %.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Frais portuaires Lomé, THC, transit maritime</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>450000</v>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>À confirmer par le transitaire.</t>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Frais portuaires, THC, transit maritime</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>INDEX(Corridors!$C$6:$F$6,1,'Hypothèses'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Piloté par le corridor retenu.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Transport routier Lomé → Niamey (conteneur 20')</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Corridor Lomé : ~1 300 000 F/20' vers Ouagadougou ; majoré pour Niamey (~1 250 km).</t>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Transport routier port → Niamey (conteneur 20')</t>
+        </is>
+      </c>
+      <c r="B16" s="12">
+        <f>INDEX(Corridors!$C$7:$F$7,1,'Hypothèses'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Piloté par le corridor retenu.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Transit, dédouanement et manutention à Niamey</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>350000</v>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Honoraires transitaire + frais de dossier.</t>
+      <c r="B17" s="12">
+        <f>INDEX(Corridors!$C$8:$F$8,1,'Hypothèses'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Piloté par le corridor retenu.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Inspection avant embarquement (% du FOB)</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="13" t="n">
         <v>0.01</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Programme de vérification des importations (COTECNA).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Frais bancaires et transfert international (% du FOB)</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="13" t="n">
         <v>0.015</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Ouverture de dossier, commissions, 50 % d'acompte TT.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Stockage et manutention magasin Niamey</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="14" t="n">
         <v>200000</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Déchargement, mise en magasin, calage.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Provision SAV et garantie 1 an (% du revient)</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="13" t="n">
         <v>0.02</v>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Pièces d'usure et interventions sous garantie.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>4. DROITS ET TAXES À L'IMPORT — NIGER (TEC UEMOA/CEDEAO), base CAF</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Droit de douane (DD) — catégorie 1, biens d'équipement</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="13" t="n">
         <v>0.05</v>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Machines agricoles SH 8433/8436/8479 : catégorie 1 = 5 %. À FAIRE CONFIRMER par le transitaire.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Redevance statistique (RS)</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B25" s="13" t="n">
         <v>0.01</v>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Prélèvement communautaire de solidarité (PCS-UEMOA)</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C26" s="7" t="inlineStr"/>
+      <c r="B26" s="13" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0,8 % appliqué au Niger (1 % dans certains États membres).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Prélèvement communautaire (PC-CEDEAO)</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="13" t="n">
         <v>0.005</v>
       </c>
-      <c r="C27" s="7" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>TVA à l'import (récupérable)</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="13" t="n">
         <v>0.19</v>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Taux de droit commun au Niger. Récupérable : hors prix de revient.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Acompte ISB/AIB (imputable)</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B29" s="13" t="n">
         <v>0.02</v>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Imputable sur l'impôt sur les bénéfices : hors prix de revient.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>5. POLITIQUE DE PRIX (coefficient appliqué au prix de revient)</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Scénario PRUDENT</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="10" t="n">
         <v>1.45</v>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Prix d'attaque / marchés à forte concurrence.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Scénario CONSEILLÉ</t>
         </is>
       </c>
-      <c r="B33" s="8" t="n">
+      <c r="B33" s="10" t="n">
         <v>1.7</v>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Positionnement de référence, cohérent avec le marché ouest-africain.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Scénario PREMIUM</t>
         </is>
       </c>
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="10" t="n">
         <v>1.9</v>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Vente à l'unité, avec installation, formation et SAV.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Arrondi commercial des prix de vente (FCFA)</t>
         </is>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Les prix de vente sont arrondis à ce multiple.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>SOURCES ET AVERTISSEMENTS</t>
         </is>
@@ -1028,6 +1080,295 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COMPARAISON DES CORRIDORS D'ACHEMINEMENT VERS NIAMEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Le scénario retenu se choisit dans l'onglet Hypothèses (cellule B3). Les montants sont des fourchettes de marché : à remplacer par la cotation ferme du transitaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Poste de coût</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>1 — LOMÉ
+(prudent)</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>2 — LOMÉ
+(optimiste)</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>3 — COTONOU via Nigeria
+(prudent)</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>4 — COTONOU frontière ouverte
+(optimiste)</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Fret maritime Qingdao → port, 20' FCL (USD)</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>1900</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>Marché 2026 Chine → Afrique de l'Ouest : 1 350 à 1 950 USD port à port.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Frais portuaires, THC, transit maritime (FCFA)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>350000</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Fourchette observée : 200 000 à 500 000 F selon le port et le transitaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Transport routier port → Niamey (FCFA)</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Fourchette 800 000 à 1 500 000 F en direct ; majorée pour le détour par le Nigeria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Transit, dédouanement et manutention Niamey (FCFA)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>Honoraires transitaire, escorte douanière, frais de dossier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Distance routière port → Niamey (km)</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>1250</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>1030</v>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Lomé–Niamey ~1 250 km ; Cotonou–Malanville–Niamey ~1 030 km ; détour Nigeria ~1 600 km.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Délai total porte à porte (jours)</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>90</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>80</v>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>Fabrication 15 j + mer 40 à 45 j + route et dédouanement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>SITUATION DU CORRIDOR BÉNIN–NIGER (août 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>• La frontière terrestre Bénin–Niger (Malanville–Gaya) est FERMÉE depuis juillet 2023 et ne l'était toujours pas rouverte en août 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>• Un accord de principe de réouverture a été acté à Niamey le 2 juin 2026 ; un comité d'experts a été installé, mais la réouverture n'est pas effective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>• Le corridor Tsamiya–Kamba, reliant le Bénin au Niger par le Nigeria, a été rouvert le 9 février 2026 : il permet d'acheminer par Cotonou, avec un détour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>• CONSÉQUENCE : tant que Malanville–Gaya reste fermé, le corridor de LOMÉ (Togo–Burkina–Niger) reste la voie la plus sûre. Le scénario 4 ne s'appliquera qu'après réouverture effective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>• À vérifier auprès du transitaire au moment de la commande : état de la frontière, escortes obligatoires et frais de transit du Nigeria le cas échéant.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1082,171 +1423,171 @@
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Modèle</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>PU FOB
 (USD)</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>FOB total
 (USD)</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>FOB total
 (FCFA)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Poids
 unit. (kg)</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>Long.
 (m)</t>
         </is>
       </c>
-      <c r="J4" s="14" t="inlineStr">
+      <c r="J4" s="16" t="inlineStr">
         <is>
           <t>Larg.
 (m)</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>Haut.
 (m)</t>
         </is>
       </c>
-      <c r="L4" s="14" t="inlineStr">
+      <c r="L4" s="16" t="inlineStr">
         <is>
           <t>Volume unit.
 emballé (m³)</t>
         </is>
       </c>
-      <c r="M4" s="14" t="inlineStr">
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>Volume
 total (m³)</t>
         </is>
       </c>
-      <c r="N4" s="14" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>Poids total
 emballé (kg)</t>
         </is>
       </c>
-      <c r="O4" s="14" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Part
 volume</t>
         </is>
       </c>
-      <c r="P4" s="14" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr">
         <is>
           <t>Part
 valeur</t>
         </is>
       </c>
-      <c r="Q4" s="14" t="inlineStr">
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>Fret + route
 réparti (FCFA)</t>
         </is>
       </c>
-      <c r="R4" s="14" t="inlineStr">
+      <c r="R4" s="16" t="inlineStr">
         <is>
           <t>Assurance
 (FCFA)</t>
         </is>
       </c>
-      <c r="S4" s="14" t="inlineStr">
+      <c r="S4" s="16" t="inlineStr">
         <is>
           <t>VALEUR CAF
 (FCFA)</t>
         </is>
       </c>
-      <c r="T4" s="14" t="inlineStr">
+      <c r="T4" s="16" t="inlineStr">
         <is>
           <t>DD 5 %
 (FCFA)</t>
         </is>
       </c>
-      <c r="U4" s="14" t="inlineStr">
+      <c r="U4" s="16" t="inlineStr">
         <is>
           <t>RS+PCS+PC
 (FCFA)</t>
         </is>
       </c>
-      <c r="V4" s="14" t="inlineStr">
+      <c r="V4" s="16" t="inlineStr">
         <is>
           <t>Total droits
 (FCFA)</t>
         </is>
       </c>
-      <c r="W4" s="14" t="inlineStr">
+      <c r="W4" s="16" t="inlineStr">
         <is>
           <t>Autres frais
 logist. (FCFA)</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="X4" s="16" t="inlineStr">
         <is>
           <t>Sous-total
 (FCFA)</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Y4" s="16" t="inlineStr">
         <is>
           <t>Provision SAV
 (FCFA)</t>
         </is>
       </c>
-      <c r="Z4" s="14" t="inlineStr">
+      <c r="Z4" s="16" t="inlineStr">
         <is>
           <t>REVIENT TOTAL
 (FCFA)</t>
         </is>
       </c>
-      <c r="AA4" s="14" t="inlineStr">
+      <c r="AA4" s="16" t="inlineStr">
         <is>
           <t>REVIENT UNIT.
 (FCFA)</t>
         </is>
       </c>
-      <c r="AB4" s="14" t="inlineStr">
+      <c r="AB4" s="16" t="inlineStr">
         <is>
           <t>TVA récup.
 (FCFA)</t>
         </is>
       </c>
-      <c r="AC4" s="14" t="inlineStr">
+      <c r="AC4" s="16" t="inlineStr">
         <is>
           <t>ISB imput.
 (FCFA)</t>
@@ -1254,551 +1595,551 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Batteuse multifonction à céréales (riz, mil, sorgho, blé) — moteur diesel 6 CV, 400–600 kg/h, sur roues</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>ZNST400</t>
         </is>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="26" t="n">
         <v>435</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="27">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="28">
         <f>F5*'Hypothèses'!$B$5</f>
         <v/>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="H5" s="29" t="n">
         <v>120</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="30" t="n">
         <v>0.8</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="30" t="n">
         <v>1.1</v>
       </c>
-      <c r="L5" s="23">
+      <c r="L5" s="31">
         <f>I5*J5*K5*'Hypothèses'!$B$8</f>
         <v/>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="31">
         <f>D5*L5</f>
         <v/>
       </c>
-      <c r="N5" s="24">
+      <c r="N5" s="32">
         <f>D5*H5*'Hypothèses'!$B$9</f>
         <v/>
       </c>
-      <c r="O5" s="25">
+      <c r="O5" s="33">
         <f>M5/$M$9</f>
         <v/>
       </c>
-      <c r="P5" s="25">
+      <c r="P5" s="33">
         <f>G5/$G$9</f>
         <v/>
       </c>
-      <c r="Q5" s="20">
+      <c r="Q5" s="28">
         <f>('Hypothèses'!$B$13+'Hypothèses'!$B$16)*O5</f>
         <v/>
       </c>
-      <c r="R5" s="20">
+      <c r="R5" s="28">
         <f>'Hypothèses'!$B$14*($G$9+'Hypothèses'!$B$13)*P5</f>
         <v/>
       </c>
-      <c r="S5" s="20">
+      <c r="S5" s="28">
         <f>G5+Q5+R5</f>
         <v/>
       </c>
-      <c r="T5" s="20">
+      <c r="T5" s="28">
         <f>S5*'Hypothèses'!$B$24</f>
         <v/>
       </c>
-      <c r="U5" s="20">
+      <c r="U5" s="28">
         <f>S5*('Hypothèses'!$B$25+'Hypothèses'!$B$26+'Hypothèses'!$B$27)</f>
         <v/>
       </c>
-      <c r="V5" s="20">
+      <c r="V5" s="28">
         <f>T5+U5</f>
         <v/>
       </c>
-      <c r="W5" s="20">
+      <c r="W5" s="28">
         <f>('Hypothèses'!$B$15+'Hypothèses'!$B$17+'Hypothèses'!$B$20)*O5+('Hypothèses'!$B$18+'Hypothèses'!$B$19)*$G$9*P5</f>
         <v/>
       </c>
-      <c r="X5" s="20">
+      <c r="X5" s="28">
         <f>S5+V5+W5</f>
         <v/>
       </c>
-      <c r="Y5" s="20">
+      <c r="Y5" s="28">
         <f>X5*'Hypothèses'!$B$21</f>
         <v/>
       </c>
-      <c r="Z5" s="20">
+      <c r="Z5" s="28">
         <f>X5+Y5</f>
         <v/>
       </c>
-      <c r="AA5" s="20">
+      <c r="AA5" s="28">
         <f>Z5/D5</f>
         <v/>
       </c>
-      <c r="AB5" s="20">
+      <c r="AB5" s="28">
         <f>(S5+V5)*'Hypothèses'!$B$28</f>
         <v/>
       </c>
-      <c r="AC5" s="20">
+      <c r="AC5" s="28">
         <f>(S5+V5)*'Hypothèses'!$B$29</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Décortiqueuse d'arachide manuelle — 40–80 kg/h</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>ZNPS-1</t>
         </is>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="26" t="n">
         <v>87</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="27">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="28">
         <f>F6*'Hypothèses'!$B$5</f>
         <v/>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="29" t="n">
         <v>25</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="30" t="n">
         <v>0.68</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="30" t="n">
         <v>0.35</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="K6" s="30" t="n">
         <v>1.15</v>
       </c>
-      <c r="L6" s="23">
+      <c r="L6" s="31">
         <f>I6*J6*K6*'Hypothèses'!$B$8</f>
         <v/>
       </c>
-      <c r="M6" s="23">
+      <c r="M6" s="31">
         <f>D6*L6</f>
         <v/>
       </c>
-      <c r="N6" s="24">
+      <c r="N6" s="32">
         <f>D6*H6*'Hypothèses'!$B$9</f>
         <v/>
       </c>
-      <c r="O6" s="25">
+      <c r="O6" s="33">
         <f>M6/$M$9</f>
         <v/>
       </c>
-      <c r="P6" s="25">
+      <c r="P6" s="33">
         <f>G6/$G$9</f>
         <v/>
       </c>
-      <c r="Q6" s="20">
+      <c r="Q6" s="28">
         <f>('Hypothèses'!$B$13+'Hypothèses'!$B$16)*O6</f>
         <v/>
       </c>
-      <c r="R6" s="20">
+      <c r="R6" s="28">
         <f>'Hypothèses'!$B$14*($G$9+'Hypothèses'!$B$13)*P6</f>
         <v/>
       </c>
-      <c r="S6" s="20">
+      <c r="S6" s="28">
         <f>G6+Q6+R6</f>
         <v/>
       </c>
-      <c r="T6" s="20">
+      <c r="T6" s="28">
         <f>S6*'Hypothèses'!$B$24</f>
         <v/>
       </c>
-      <c r="U6" s="20">
+      <c r="U6" s="28">
         <f>S6*('Hypothèses'!$B$25+'Hypothèses'!$B$26+'Hypothèses'!$B$27)</f>
         <v/>
       </c>
-      <c r="V6" s="20">
+      <c r="V6" s="28">
         <f>T6+U6</f>
         <v/>
       </c>
-      <c r="W6" s="20">
+      <c r="W6" s="28">
         <f>('Hypothèses'!$B$15+'Hypothèses'!$B$17+'Hypothèses'!$B$20)*O6+('Hypothèses'!$B$18+'Hypothèses'!$B$19)*$G$9*P6</f>
         <v/>
       </c>
-      <c r="X6" s="20">
+      <c r="X6" s="28">
         <f>S6+V6+W6</f>
         <v/>
       </c>
-      <c r="Y6" s="20">
+      <c r="Y6" s="28">
         <f>X6*'Hypothèses'!$B$21</f>
         <v/>
       </c>
-      <c r="Z6" s="20">
+      <c r="Z6" s="28">
         <f>X6+Y6</f>
         <v/>
       </c>
-      <c r="AA6" s="20">
+      <c r="AA6" s="28">
         <f>Z6/D6</f>
         <v/>
       </c>
-      <c r="AB6" s="20">
+      <c r="AB6" s="28">
         <f>(S6+V6)*'Hypothèses'!$B$28</f>
         <v/>
       </c>
-      <c r="AC6" s="20">
+      <c r="AC6" s="28">
         <f>(S6+V6)*'Hypothèses'!$B$29</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Broyeur / moulin à céréales et résidus végétaux — moteur diesel 10 CV, cyclone, 200–400 kg/h</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>ZNGQ360</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="26" t="n">
         <v>582</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="27">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="28">
         <f>F7*'Hypothèses'!$B$5</f>
         <v/>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="29" t="n">
         <v>260</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="I7" s="30" t="n">
         <v>0.65</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="K7" s="30" t="n">
         <v>1.3</v>
       </c>
-      <c r="L7" s="23">
+      <c r="L7" s="31">
         <f>I7*J7*K7*'Hypothèses'!$B$8</f>
         <v/>
       </c>
-      <c r="M7" s="23">
+      <c r="M7" s="31">
         <f>D7*L7</f>
         <v/>
       </c>
-      <c r="N7" s="24">
+      <c r="N7" s="32">
         <f>D7*H7*'Hypothèses'!$B$9</f>
         <v/>
       </c>
-      <c r="O7" s="25">
+      <c r="O7" s="33">
         <f>M7/$M$9</f>
         <v/>
       </c>
-      <c r="P7" s="25">
+      <c r="P7" s="33">
         <f>G7/$G$9</f>
         <v/>
       </c>
-      <c r="Q7" s="20">
+      <c r="Q7" s="28">
         <f>('Hypothèses'!$B$13+'Hypothèses'!$B$16)*O7</f>
         <v/>
       </c>
-      <c r="R7" s="20">
+      <c r="R7" s="28">
         <f>'Hypothèses'!$B$14*($G$9+'Hypothèses'!$B$13)*P7</f>
         <v/>
       </c>
-      <c r="S7" s="20">
+      <c r="S7" s="28">
         <f>G7+Q7+R7</f>
         <v/>
       </c>
-      <c r="T7" s="20">
+      <c r="T7" s="28">
         <f>S7*'Hypothèses'!$B$24</f>
         <v/>
       </c>
-      <c r="U7" s="20">
+      <c r="U7" s="28">
         <f>S7*('Hypothèses'!$B$25+'Hypothèses'!$B$26+'Hypothèses'!$B$27)</f>
         <v/>
       </c>
-      <c r="V7" s="20">
+      <c r="V7" s="28">
         <f>T7+U7</f>
         <v/>
       </c>
-      <c r="W7" s="20">
+      <c r="W7" s="28">
         <f>('Hypothèses'!$B$15+'Hypothèses'!$B$17+'Hypothèses'!$B$20)*O7+('Hypothèses'!$B$18+'Hypothèses'!$B$19)*$G$9*P7</f>
         <v/>
       </c>
-      <c r="X7" s="20">
+      <c r="X7" s="28">
         <f>S7+V7+W7</f>
         <v/>
       </c>
-      <c r="Y7" s="20">
+      <c r="Y7" s="28">
         <f>X7*'Hypothèses'!$B$21</f>
         <v/>
       </c>
-      <c r="Z7" s="20">
+      <c r="Z7" s="28">
         <f>X7+Y7</f>
         <v/>
       </c>
-      <c r="AA7" s="20">
+      <c r="AA7" s="28">
         <f>Z7/D7</f>
         <v/>
       </c>
-      <c r="AB7" s="20">
+      <c r="AB7" s="28">
         <f>(S7+V7)*'Hypothèses'!$B$28</f>
         <v/>
       </c>
-      <c r="AC7" s="20">
+      <c r="AC7" s="28">
         <f>(S7+V7)*'Hypothèses'!$B$29</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="15" t="n">
+      <c r="A8" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Presse à huile motorisée inox (arachide, sésame, soja, tournesol) — électrique 4 kW, 10–30 kg/h</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>ZYSS20</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="26" t="n">
         <v>1035</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="27">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="28">
         <f>F8*'Hypothèses'!$B$5</f>
         <v/>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="29" t="n">
         <v>60</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="30" t="n">
         <v>0.82</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="30" t="n">
         <v>0.45</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="K8" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="23">
+      <c r="L8" s="31">
         <f>I8*J8*K8*'Hypothèses'!$B$8</f>
         <v/>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="31">
         <f>D8*L8</f>
         <v/>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="32">
         <f>D8*H8*'Hypothèses'!$B$9</f>
         <v/>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="33">
         <f>M8/$M$9</f>
         <v/>
       </c>
-      <c r="P8" s="25">
+      <c r="P8" s="33">
         <f>G8/$G$9</f>
         <v/>
       </c>
-      <c r="Q8" s="20">
+      <c r="Q8" s="28">
         <f>('Hypothèses'!$B$13+'Hypothèses'!$B$16)*O8</f>
         <v/>
       </c>
-      <c r="R8" s="20">
+      <c r="R8" s="28">
         <f>'Hypothèses'!$B$14*($G$9+'Hypothèses'!$B$13)*P8</f>
         <v/>
       </c>
-      <c r="S8" s="20">
+      <c r="S8" s="28">
         <f>G8+Q8+R8</f>
         <v/>
       </c>
-      <c r="T8" s="20">
+      <c r="T8" s="28">
         <f>S8*'Hypothèses'!$B$24</f>
         <v/>
       </c>
-      <c r="U8" s="20">
+      <c r="U8" s="28">
         <f>S8*('Hypothèses'!$B$25+'Hypothèses'!$B$26+'Hypothèses'!$B$27)</f>
         <v/>
       </c>
-      <c r="V8" s="20">
+      <c r="V8" s="28">
         <f>T8+U8</f>
         <v/>
       </c>
-      <c r="W8" s="20">
+      <c r="W8" s="28">
         <f>('Hypothèses'!$B$15+'Hypothèses'!$B$17+'Hypothèses'!$B$20)*O8+('Hypothèses'!$B$18+'Hypothèses'!$B$19)*$G$9*P8</f>
         <v/>
       </c>
-      <c r="X8" s="20">
+      <c r="X8" s="28">
         <f>S8+V8+W8</f>
         <v/>
       </c>
-      <c r="Y8" s="20">
+      <c r="Y8" s="28">
         <f>X8*'Hypothèses'!$B$21</f>
         <v/>
       </c>
-      <c r="Z8" s="20">
+      <c r="Z8" s="28">
         <f>X8+Y8</f>
         <v/>
       </c>
-      <c r="AA8" s="20">
+      <c r="AA8" s="28">
         <f>Z8/D8</f>
         <v/>
       </c>
-      <c r="AB8" s="20">
+      <c r="AB8" s="28">
         <f>(S8+V8)*'Hypothèses'!$B$28</f>
         <v/>
       </c>
-      <c r="AC8" s="20">
+      <c r="AC8" s="28">
         <f>(S8+V8)*'Hypothèses'!$B$29</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="n"/>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="A9" s="34" t="n"/>
+      <c r="B9" s="34" t="inlineStr">
         <is>
           <t>TOTAL / CONTENEUR 20'</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n"/>
-      <c r="D9" s="26">
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="34">
         <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27">
+      <c r="E9" s="35" t="n"/>
+      <c r="F9" s="35">
         <f>SUM(F5:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="36">
         <f>SUM(G5:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="29" t="n"/>
-      <c r="I9" s="30" t="n"/>
-      <c r="J9" s="30" t="n"/>
-      <c r="K9" s="30" t="n"/>
-      <c r="L9" s="30" t="n"/>
-      <c r="M9" s="30">
+      <c r="H9" s="37" t="n"/>
+      <c r="I9" s="38" t="n"/>
+      <c r="J9" s="38" t="n"/>
+      <c r="K9" s="38" t="n"/>
+      <c r="L9" s="38" t="n"/>
+      <c r="M9" s="38">
         <f>SUM(M5:M8)</f>
         <v/>
       </c>
-      <c r="N9" s="31">
+      <c r="N9" s="39">
         <f>SUM(N5:N8)</f>
         <v/>
       </c>
-      <c r="O9" s="32">
+      <c r="O9" s="40">
         <f>SUM(O5:O8)</f>
         <v/>
       </c>
-      <c r="P9" s="32">
+      <c r="P9" s="40">
         <f>SUM(P5:P8)</f>
         <v/>
       </c>
-      <c r="Q9" s="28">
+      <c r="Q9" s="36">
         <f>SUM(Q5:Q8)</f>
         <v/>
       </c>
-      <c r="R9" s="28">
+      <c r="R9" s="36">
         <f>SUM(R5:R8)</f>
         <v/>
       </c>
-      <c r="S9" s="28">
+      <c r="S9" s="36">
         <f>SUM(S5:S8)</f>
         <v/>
       </c>
-      <c r="T9" s="28">
+      <c r="T9" s="36">
         <f>SUM(T5:T8)</f>
         <v/>
       </c>
-      <c r="U9" s="28">
+      <c r="U9" s="36">
         <f>SUM(U5:U8)</f>
         <v/>
       </c>
-      <c r="V9" s="28">
+      <c r="V9" s="36">
         <f>SUM(V5:V8)</f>
         <v/>
       </c>
-      <c r="W9" s="28">
+      <c r="W9" s="36">
         <f>SUM(W5:W8)</f>
         <v/>
       </c>
-      <c r="X9" s="28">
+      <c r="X9" s="36">
         <f>SUM(X5:X8)</f>
         <v/>
       </c>
-      <c r="Y9" s="28">
+      <c r="Y9" s="36">
         <f>SUM(Y5:Y8)</f>
         <v/>
       </c>
-      <c r="Z9" s="28">
+      <c r="Z9" s="36">
         <f>SUM(Z5:Z8)</f>
         <v/>
       </c>
-      <c r="AA9" s="28" t="n"/>
-      <c r="AB9" s="28">
+      <c r="AA9" s="36" t="n"/>
+      <c r="AB9" s="36">
         <f>SUM(AB5:AB8)</f>
         <v/>
       </c>
-      <c r="AC9" s="28">
+      <c r="AC9" s="36">
         <f>SUM(AC5:AC8)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>LÉGENDE</t>
         </is>
@@ -1837,7 +2178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1878,87 +2219,87 @@
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Modèle</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Prix de revient
 unitaire (FCFA)</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>PV HT PRUDENT
 (FCFA)</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>PV HT CONSEILLÉ
 (FCFA)</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>PV HT PREMIUM
 (FCFA)</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>PV TTC conseillé
 (FCFA)</t>
         </is>
       </c>
-      <c r="J4" s="14" t="inlineStr">
+      <c r="J4" s="16" t="inlineStr">
         <is>
           <t>Marge unitaire
 conseillée (FCFA)</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>Taux de marge
 / PV HT</t>
         </is>
       </c>
-      <c r="L4" s="14" t="inlineStr">
+      <c r="L4" s="16" t="inlineStr">
         <is>
           <t>Repère marché
 Afr. Ouest (FCFA)</t>
         </is>
       </c>
-      <c r="M4" s="14" t="inlineStr">
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>Position vs
 marché</t>
         </is>
       </c>
-      <c r="N4" s="14" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>CA HT conseillé
 sur 10 unités</t>
         </is>
       </c>
-      <c r="O4" s="14" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Marge brute
 sur 10 unités</t>
@@ -1966,284 +2307,284 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="33" t="n">
+      <c r="A5" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>Batteuse multifonction à céréales — diesel 6 CV</t>
         </is>
       </c>
-      <c r="C5" s="35">
+      <c r="C5" s="43">
         <f>'Prix de revient'!C5</f>
         <v/>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="43">
         <f>'Prix de revient'!D5</f>
         <v/>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="44">
         <f>'Prix de revient'!AA5</f>
         <v/>
       </c>
-      <c r="F5" s="37">
+      <c r="F5" s="45">
         <f>ROUND(E5*'Hypothèses'!$B$32/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="G5" s="37">
+      <c r="G5" s="45">
         <f>ROUND(E5*'Hypothèses'!$B$33/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="H5" s="37">
+      <c r="H5" s="45">
         <f>ROUND(E5*'Hypothèses'!$B$34/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="I5" s="37">
+      <c r="I5" s="45">
         <f>G5*(1+'Hypothèses'!$B$28)</f>
         <v/>
       </c>
-      <c r="J5" s="37">
+      <c r="J5" s="45">
         <f>G5-E5</f>
         <v/>
       </c>
-      <c r="K5" s="38">
+      <c r="K5" s="46">
         <f>IF(G5=0,0,(G5-E5)/G5)</f>
         <v/>
       </c>
-      <c r="L5" s="39" t="n">
+      <c r="L5" s="20" t="n">
         <v>950000</v>
       </c>
-      <c r="M5" s="38">
+      <c r="M5" s="46">
         <f>IF(L5=0,0,G5/L5-1)</f>
         <v/>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="45">
         <f>D5*G5</f>
         <v/>
       </c>
-      <c r="O5" s="37">
+      <c r="O5" s="45">
         <f>D5*(G5-E5)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="33" t="n">
+      <c r="A6" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="34" t="inlineStr">
+      <c r="B6" s="42" t="inlineStr">
         <is>
           <t>Décortiqueuse d'arachide manuelle</t>
         </is>
       </c>
-      <c r="C6" s="35">
+      <c r="C6" s="43">
         <f>'Prix de revient'!C6</f>
         <v/>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="43">
         <f>'Prix de revient'!D6</f>
         <v/>
       </c>
-      <c r="E6" s="36">
+      <c r="E6" s="44">
         <f>'Prix de revient'!AA6</f>
         <v/>
       </c>
-      <c r="F6" s="37">
+      <c r="F6" s="45">
         <f>ROUND(E6*'Hypothèses'!$B$32/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="G6" s="37">
+      <c r="G6" s="45">
         <f>ROUND(E6*'Hypothèses'!$B$33/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="H6" s="37">
+      <c r="H6" s="45">
         <f>ROUND(E6*'Hypothèses'!$B$34/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="I6" s="37">
+      <c r="I6" s="45">
         <f>G6*(1+'Hypothèses'!$B$28)</f>
         <v/>
       </c>
-      <c r="J6" s="37">
+      <c r="J6" s="45">
         <f>G6-E6</f>
         <v/>
       </c>
-      <c r="K6" s="38">
+      <c r="K6" s="46">
         <f>IF(G6=0,0,(G6-E6)/G6)</f>
         <v/>
       </c>
-      <c r="L6" s="39" t="n">
+      <c r="L6" s="20" t="n">
         <v>200000</v>
       </c>
-      <c r="M6" s="38">
+      <c r="M6" s="46">
         <f>IF(L6=0,0,G6/L6-1)</f>
         <v/>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="45">
         <f>D6*G6</f>
         <v/>
       </c>
-      <c r="O6" s="37">
+      <c r="O6" s="45">
         <f>D6*(G6-E6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="33" t="n">
+      <c r="A7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Broyeur / moulin à céréales — diesel 10 CV</t>
         </is>
       </c>
-      <c r="C7" s="35">
+      <c r="C7" s="43">
         <f>'Prix de revient'!C7</f>
         <v/>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="43">
         <f>'Prix de revient'!D7</f>
         <v/>
       </c>
-      <c r="E7" s="36">
+      <c r="E7" s="44">
         <f>'Prix de revient'!AA7</f>
         <v/>
       </c>
-      <c r="F7" s="37">
+      <c r="F7" s="45">
         <f>ROUND(E7*'Hypothèses'!$B$32/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="G7" s="37">
+      <c r="G7" s="45">
         <f>ROUND(E7*'Hypothèses'!$B$33/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="H7" s="37">
+      <c r="H7" s="45">
         <f>ROUND(E7*'Hypothèses'!$B$34/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="I7" s="37">
+      <c r="I7" s="45">
         <f>G7*(1+'Hypothèses'!$B$28)</f>
         <v/>
       </c>
-      <c r="J7" s="37">
+      <c r="J7" s="45">
         <f>G7-E7</f>
         <v/>
       </c>
-      <c r="K7" s="38">
+      <c r="K7" s="46">
         <f>IF(G7=0,0,(G7-E7)/G7)</f>
         <v/>
       </c>
-      <c r="L7" s="39" t="n">
+      <c r="L7" s="20" t="n">
         <v>850000</v>
       </c>
-      <c r="M7" s="38">
+      <c r="M7" s="46">
         <f>IF(L7=0,0,G7/L7-1)</f>
         <v/>
       </c>
-      <c r="N7" s="37">
+      <c r="N7" s="45">
         <f>D7*G7</f>
         <v/>
       </c>
-      <c r="O7" s="37">
+      <c r="O7" s="45">
         <f>D7*(G7-E7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="33" t="n">
+      <c r="A8" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="42" t="inlineStr">
         <is>
           <t>Presse à huile motorisée inox — 4 kW</t>
         </is>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="43">
         <f>'Prix de revient'!C8</f>
         <v/>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="43">
         <f>'Prix de revient'!D8</f>
         <v/>
       </c>
-      <c r="E8" s="36">
+      <c r="E8" s="44">
         <f>'Prix de revient'!AA8</f>
         <v/>
       </c>
-      <c r="F8" s="37">
+      <c r="F8" s="45">
         <f>ROUND(E8*'Hypothèses'!$B$32/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="G8" s="37">
+      <c r="G8" s="45">
         <f>ROUND(E8*'Hypothèses'!$B$33/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="H8" s="37">
+      <c r="H8" s="45">
         <f>ROUND(E8*'Hypothèses'!$B$34/'Hypothèses'!$B$35,0)*'Hypothèses'!$B$35</f>
         <v/>
       </c>
-      <c r="I8" s="37">
+      <c r="I8" s="45">
         <f>G8*(1+'Hypothèses'!$B$28)</f>
         <v/>
       </c>
-      <c r="J8" s="37">
+      <c r="J8" s="45">
         <f>G8-E8</f>
         <v/>
       </c>
-      <c r="K8" s="38">
+      <c r="K8" s="46">
         <f>IF(G8=0,0,(G8-E8)/G8)</f>
         <v/>
       </c>
-      <c r="L8" s="39" t="n">
+      <c r="L8" s="20" t="n">
         <v>1300000</v>
       </c>
-      <c r="M8" s="38">
+      <c r="M8" s="46">
         <f>IF(L8=0,0,G8/L8-1)</f>
         <v/>
       </c>
-      <c r="N8" s="37">
+      <c r="N8" s="45">
         <f>D8*G8</f>
         <v/>
       </c>
-      <c r="O8" s="37">
+      <c r="O8" s="45">
         <f>D8*(G8-E8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="n"/>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="A9" s="34" t="n"/>
+      <c r="B9" s="34" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n"/>
-      <c r="D9" s="26">
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="34">
         <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
-      <c r="H9" s="28" t="n"/>
-      <c r="I9" s="28" t="n"/>
-      <c r="J9" s="28" t="n"/>
-      <c r="K9" s="32">
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="36" t="n"/>
+      <c r="G9" s="36" t="n"/>
+      <c r="H9" s="36" t="n"/>
+      <c r="I9" s="36" t="n"/>
+      <c r="J9" s="36" t="n"/>
+      <c r="K9" s="40">
         <f>IF(N9=0,0,O9/N9)</f>
         <v/>
       </c>
-      <c r="L9" s="28" t="n"/>
-      <c r="M9" s="32" t="n"/>
-      <c r="N9" s="28">
+      <c r="L9" s="36" t="n"/>
+      <c r="M9" s="40" t="n"/>
+      <c r="N9" s="36">
         <f>SUM(N5:N8)</f>
         <v/>
       </c>
-      <c r="O9" s="28">
+      <c r="O9" s="36">
         <f>SUM(O5:O8)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>LECTURE</t>
         </is>
@@ -2289,7 +2630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2311,412 +2652,411 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>A. DÉCAISSEMENTS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Achat marchandise FOB Qingdao</t>
         </is>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="12">
         <f>'Prix de revient'!G9</f>
         <v/>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>50 % d'acompte à la commande, solde avant expédition.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Fret, assurance, transport et frais logistiques</t>
         </is>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="12">
         <f>'Prix de revient'!Q9+'Prix de revient'!R9+'Prix de revient'!W9</f>
         <v/>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Droits et taxes de douane (non récupérables)</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="12">
         <f>'Prix de revient'!V9</f>
         <v/>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>DD + RS + PCS + PC sur la valeur CAF.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Provision SAV et garantie</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="12">
         <f>'Prix de revient'!Y9</f>
         <v/>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>PRIX DE REVIENT TOTAL HT (rendu magasin Niamey)</t>
         </is>
       </c>
-      <c r="B8" s="41">
+      <c r="B8" s="48">
         <f>'Prix de revient'!Z9</f>
         <v/>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>Base de calcul des prix de vente.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>TVA à l'import (récupérable)</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="12">
         <f>'Prix de revient'!AB9</f>
         <v/>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Récupérée sur la TVA collectée à la vente.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Acompte ISB 2 % (imputable)</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="12">
         <f>'Prix de revient'!AC9</f>
         <v/>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Imputable sur l'impôt sur les bénéfices.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="50" t="inlineStr">
         <is>
           <t>TRÉSORERIE À MOBILISER (toutes taxes comprises)</t>
         </is>
       </c>
-      <c r="B11" s="44">
+      <c r="B11" s="51">
         <f>B8+B9+B10</f>
         <v/>
       </c>
-      <c r="C11" s="45" t="inlineStr">
+      <c r="C11" s="52" t="inlineStr">
         <is>
           <t>Montant réellement à financer jusqu'à la revente.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>B. CHIFFRE D'AFFAIRES ET MARGE (40 machines vendues)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Chiffre d'affaires HT — scénario PRUDENT</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="12">
         <f>SUMPRODUCT('Prix de vente'!D5:D8,'Prix de vente'!F5:F8)</f>
         <v/>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
+      <c r="C14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>Chiffre d'affaires HT — scénario CONSEILLÉ</t>
         </is>
       </c>
-      <c r="B15" s="47">
+      <c r="B15" s="54">
         <f>SUMPRODUCT('Prix de vente'!D5:D8,'Prix de vente'!G5:G8)</f>
         <v/>
       </c>
-      <c r="C15" s="7" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Chiffre d'affaires HT — scénario PREMIUM</t>
         </is>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="12">
         <f>SUMPRODUCT('Prix de vente'!D5:D8,'Prix de vente'!H5:H8)</f>
         <v/>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Marge brute — scénario PRUDENT</t>
         </is>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="12">
         <f>B14-B8</f>
         <v/>
       </c>
-      <c r="C17" s="7" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="40" t="inlineStr">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>Marge brute — scénario CONSEILLÉ</t>
         </is>
       </c>
-      <c r="B18" s="41">
+      <c r="B18" s="48">
         <f>B15-B8</f>
         <v/>
       </c>
-      <c r="C18" s="42" t="inlineStr"/>
+      <c r="C18" s="49" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Marge brute — scénario PREMIUM</t>
         </is>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="12">
         <f>B16-B8</f>
         <v/>
       </c>
-      <c r="C19" s="7" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Taux de marge sur CA — scénario CONSEILLÉ</t>
         </is>
       </c>
-      <c r="B20" s="48">
+      <c r="B20" s="55">
         <f>IF(B15=0,0,B18/B15)</f>
         <v/>
       </c>
-      <c r="C20" s="7" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Rentabilité de l'investissement — scénario CONSEILLÉ</t>
         </is>
       </c>
-      <c r="B21" s="48">
+      <c r="B21" s="55">
         <f>IF(B8=0,0,B18/B8)</f>
         <v/>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Marge brute rapportée au prix de revient engagé.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>C. LOGISTIQUE DE L'OPÉRATION</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Volume total emballé</t>
         </is>
       </c>
-      <c r="B24" s="49">
+      <c r="B24" s="56">
         <f>'Prix de revient'!M9</f>
         <v/>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Conteneur 20' : ~33 m³ — chargement possible.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Poids total emballé (kg)</t>
         </is>
       </c>
-      <c r="B25" s="50">
+      <c r="B25" s="57">
         <f>'Prix de revient'!N9</f>
         <v/>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Conteneur 20' : 28 t de charge utile.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Nombre de machines</t>
         </is>
       </c>
-      <c r="B26" s="50">
+      <c r="B26" s="57">
         <f>'Prix de revient'!D9</f>
         <v/>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>4 modèles × 10 unités (MOQ du fournisseur).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>D. DÉLAI PRÉVISIONNEL</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Fabrication après paiement de l'acompte</t>
         </is>
       </c>
-      <c r="B29" s="51" t="inlineStr">
+      <c r="B29" s="58" t="inlineStr">
         <is>
           <t>15 jours</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Transport maritime Qingdao → Lomé</t>
         </is>
       </c>
-      <c r="B30" s="51" t="inlineStr">
+      <c r="B30" s="58" t="inlineStr">
         <is>
           <t>40 à 45 jours</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Déchargement, transit et route Lomé → Niamey</t>
         </is>
       </c>
-      <c r="B31" s="51" t="inlineStr">
+      <c r="B31" s="58" t="inlineStr">
         <is>
           <t>12 à 18 jours</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Dédouanement et mise en magasin à Niamey</t>
         </is>
       </c>
-      <c r="B32" s="51" t="inlineStr">
+      <c r="B32" s="58" t="inlineStr">
         <is>
           <t>5 à 8 jours</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="46" t="inlineStr">
-        <is>
-          <t>DÉLAI TOTAL ESTIMÉ</t>
-        </is>
-      </c>
-      <c r="B33" s="52" t="inlineStr">
-        <is>
-          <t>environ 75 à 90 jours</t>
-        </is>
+      <c r="A33" s="53" t="inlineStr">
+        <is>
+          <t>DÉLAI TOTAL ESTIMÉ (corridor retenu)</t>
+        </is>
+      </c>
+      <c r="B33" s="59">
+        <f>INDEX(Corridors!$C$10:$F$10,1,'Hypothèses'!$B$3)&amp;" jours"</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>E. POINTS À VÉRIFIER AVANT ENGAGEMENT</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="53" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>• Classement tarifaire exact (SH) de chaque machine et catégorie du TEC : confirmer le taux de 5 % auprès du transitaire.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="53" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>• Existence d'une exonération ou d'un régime de faveur pour le matériel agricole (Code des investissements, projets financés).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="53" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>• Cotation ferme du transitaire : fret maritime, frais portuaires de Lomé, transport routier, transit et dédouanement.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="53" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>• Coût réel du transfert bancaire et disponibilité des devises pour l'acompte de 50 %.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="53" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>• Relevé des prix réellement pratiqués à Niamey pour ces quatre familles de machines.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="53" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>• Disponibilité des pièces d'usure (tamis, courroies, marteaux, vis de presse) : à commander avec la machine.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="53" t="inlineStr">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>• Norme électrique de la presse à huile (4 kW) : vérifier la compatibilité 220 V / 380 V avec le réseau du client.</t>
         </is>

</xml_diff>